<commit_message>
Login and Register TestCases
</commit_message>
<xml_diff>
--- a/TestCases_Docs/Login_Tcs.xlsx
+++ b/TestCases_Docs/Login_Tcs.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yasse\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yasse\OneDrive\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29C3F9DA-C9F8-400F-A65E-E6D2532EF4AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC9D08BE-6031-42A2-B0D6-45FEADE4866C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="757" uniqueCount="337">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="757" uniqueCount="338">
   <si>
     <t>TesTCASE ID</t>
   </si>
@@ -1510,6 +1510,9 @@
   <si>
     <t>SIQ_Acc_09</t>
   </si>
+  <si>
+    <t>SRS-FN-login-004</t>
+  </si>
 </sst>
 </file>
 
@@ -2109,22 +2112,6 @@
       </fill>
     </dxf>
     <dxf>
-      <border>
-        <left style="thin">
-          <color rgb="FF356854"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF356854"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF356854"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF356854"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFF6F8F9"/>
@@ -2148,13 +2135,29 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF356854"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF356854"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF356854"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF356854"/>
+        </bottom>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="18">
     <tableStyle name="Register_Tcs-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="34"/>
-      <tableStyleElement type="headerRow" dxfId="37"/>
-      <tableStyleElement type="firstRowStripe" dxfId="36"/>
-      <tableStyleElement type="secondRowStripe" dxfId="35"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="37"/>
+      <tableStyleElement type="headerRow" dxfId="36"/>
+      <tableStyleElement type="firstRowStripe" dxfId="35"/>
+      <tableStyleElement type="secondRowStripe" dxfId="34"/>
     </tableStyle>
     <tableStyle name="Register_Tcs-style 2" pivot="0" count="2" xr9:uid="{00000000-0011-0000-FFFF-FFFF01000000}">
       <tableStyleElement type="firstRowStripe" dxfId="33"/>
@@ -2989,7 +2992,7 @@
       <c r="K4" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="L4" s="2" t="s">
+      <c r="L4" s="3" t="s">
         <v>39</v>
       </c>
       <c r="M4" s="2" t="s">
@@ -3049,7 +3052,7 @@
         <v>17</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>31</v>
+        <v>337</v>
       </c>
       <c r="M5" s="2" t="s">
         <v>20</v>
@@ -3108,7 +3111,7 @@
         <v>17</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>31</v>
+        <v>337</v>
       </c>
       <c r="M6" s="2" t="s">
         <v>20</v>
@@ -3167,7 +3170,7 @@
         <v>17</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>31</v>
+        <v>337</v>
       </c>
       <c r="M7" s="2" t="s">
         <v>20</v>

</xml_diff>

<commit_message>
test/refactor Login Test cases
</commit_message>
<xml_diff>
--- a/TestCases_Docs/Login_Tcs.xlsx
+++ b/TestCases_Docs/Login_Tcs.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="802" uniqueCount="357">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="802" uniqueCount="358">
   <si>
     <t>TesTCASE ID</t>
   </si>
@@ -120,7 +120,7 @@
  3. Type a valid Email</t>
   </si>
   <si>
-    <t xml:space="preserve"> Email = fatma@gmail.com</t>
+    <t xml:space="preserve"> Email = fatma123@gmail.com</t>
   </si>
   <si>
     <t xml:space="preserve"> 1. Email field is displayed   
@@ -145,7 +145,7 @@
  3. Type a valid Password</t>
   </si>
   <si>
-    <t>Password = Pass@1234</t>
+    <t>Password = Pass@123</t>
   </si>
   <si>
     <t xml:space="preserve"> 1. Password field is displayed   
@@ -180,7 +180,7 @@
     <t>TC-Login-005</t>
   </si>
   <si>
-    <t>Verify that user can successfully login as Client with valid credentials.</t>
+    <t>Verify that user can successfully login as Customer with valid credentials.</t>
   </si>
   <si>
     <t>1.User is on Home page 
@@ -194,15 +194,15 @@
  3. Click Submit button</t>
   </si>
   <si>
-    <t xml:space="preserve">1.fatma@gmail.com
-2.pass@1234
+    <t xml:space="preserve">1.fatma123@gmail.com
+2.pass@123
 </t>
   </si>
   <si>
     <t xml:space="preserve">User is redirected to Home page </t>
   </si>
   <si>
-    <t>User is logged in as Client.</t>
+    <t>User is logged in as Customer .</t>
   </si>
   <si>
     <t>SRS-FN-login-001,
@@ -299,7 +299,7 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">1.fatma@gmail.com
+    <t xml:space="preserve">1.fatma123@gmail.com
  2. Leave Password empty 
 </t>
   </si>
@@ -348,7 +348,7 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">1. fatma@gmail.com
+    <t xml:space="preserve">1. fatma123@gmail.com
  2. Password=123456767
 </t>
   </si>
@@ -381,7 +381,7 @@
   </si>
   <si>
     <t xml:space="preserve">1. tweety@gmail.com
- 2. Password=pass@1234
+ 2. Password=pass@123
 </t>
   </si>
   <si>
@@ -415,6 +415,9 @@
 2. Observe the field while typing and after typing</t>
   </si>
   <si>
+    <t>Password = Pass@1234</t>
+  </si>
+  <si>
     <t>Password appears as dots and not as plain text</t>
   </si>
   <si>
@@ -467,8 +470,8 @@
 3. Check the URL after submission</t>
   </si>
   <si>
-    <t>Email=fatma@gmail.com
-Password=pass@1234</t>
+    <t>Email=fatma123@gmail.com
+Password=pass@123</t>
   </si>
   <si>
     <t>URL does NOT contain email or password parameters .</t>
@@ -2871,7 +2874,7 @@
       <c r="A6" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="9" t="s">
         <v>50</v>
       </c>
       <c r="C6" s="3" t="s">
@@ -2886,13 +2889,13 @@
       <c r="F6" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="G6" s="5" t="s">
+      <c r="G6" s="10" t="s">
         <v>53</v>
       </c>
       <c r="H6" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="I6" s="4" t="s">
+      <c r="I6" s="9" t="s">
         <v>55</v>
       </c>
       <c r="J6" s="6" t="s">
@@ -3122,7 +3125,7 @@
       <c r="F10" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="G10" s="5" t="s">
+      <c r="G10" s="10" t="s">
         <v>80</v>
       </c>
       <c r="H10" s="4" t="s">
@@ -3240,7 +3243,7 @@
       <c r="F12" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="G12" s="5" t="s">
+      <c r="G12" s="10" t="s">
         <v>91</v>
       </c>
       <c r="H12" s="4" t="s">
@@ -3299,7 +3302,7 @@
       <c r="F13" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="G13" s="5" t="s">
+      <c r="G13" s="10" t="s">
         <v>98</v>
       </c>
       <c r="H13" s="4" t="s">
@@ -3418,13 +3421,13 @@
         <v>106</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>40</v>
+        <v>107</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="J15" s="6" t="s">
         <v>24</v>
@@ -3459,10 +3462,10 @@
     </row>
     <row r="16" ht="69.0" customHeight="1">
       <c r="A16" s="8" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C16" s="3" t="s">
         <v>17</v>
@@ -3474,16 +3477,16 @@
         <v>96</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>40</v>
+        <v>107</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J16" s="6" t="s">
         <v>24</v>
@@ -3518,10 +3521,10 @@
     </row>
     <row r="17" ht="69.0" customHeight="1">
       <c r="A17" s="8" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>17</v>
@@ -3533,16 +3536,16 @@
         <v>96</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="G17" s="5" t="s">
         <v>21</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="I17" s="4" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="J17" s="6" t="s">
         <v>24</v>
@@ -3577,10 +3580,10 @@
     </row>
     <row r="18" ht="69.0" customHeight="1">
       <c r="A18" s="8" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>17</v>
@@ -3592,16 +3595,16 @@
         <v>96</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>121</v>
-      </c>
-      <c r="G18" s="5" t="s">
         <v>122</v>
       </c>
+      <c r="G18" s="10" t="s">
+        <v>123</v>
+      </c>
       <c r="H18" s="4" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I18" s="4" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="J18" s="6" t="s">
         <v>24</v>
@@ -4803,7 +4806,7 @@
       <c r="D59" s="2"/>
       <c r="E59" s="2"/>
       <c r="F59" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G59" s="2"/>
       <c r="H59" s="22"/>
@@ -11434,7 +11437,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
@@ -11449,7 +11452,7 @@
         <v>7</v>
       </c>
       <c r="I1" s="40" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>8</v>
@@ -11473,54 +11476,54 @@
         <v>14</v>
       </c>
       <c r="Q1" s="40" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="2" ht="99.0" customHeight="1">
       <c r="A2" s="41" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B2" s="42" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C2" s="41" t="s">
         <v>17</v>
       </c>
       <c r="D2" s="41" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E2" s="43" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F2" s="42" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G2" s="42" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H2" s="41" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="I2" s="42" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="J2" s="41"/>
       <c r="K2" s="41" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L2" s="41"/>
       <c r="M2" s="41" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="N2" s="41" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="O2" s="41" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="P2" s="41"/>
       <c r="Q2" s="41" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="R2" s="41"/>
       <c r="S2" s="41"/>
@@ -11537,49 +11540,49 @@
     </row>
     <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="41" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B3" s="42" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C3" s="41" t="s">
         <v>71</v>
       </c>
       <c r="D3" s="41" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E3" s="43" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F3" s="42" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="G3" s="41" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="H3" s="42" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="I3" s="42" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="J3" s="41"/>
       <c r="K3" s="41" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L3" s="41"/>
       <c r="M3" s="41" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="N3" s="41" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="O3" s="41" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="P3" s="41"/>
       <c r="Q3" s="41" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="R3" s="41"/>
       <c r="S3" s="41"/>
@@ -11596,49 +11599,49 @@
     </row>
     <row r="4" ht="15.75" customHeight="1">
       <c r="A4" s="41" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B4" s="42" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C4" s="41" t="s">
         <v>71</v>
       </c>
       <c r="D4" s="41" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E4" s="43" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F4" s="42" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="G4" s="42" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="H4" s="42" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="I4" s="42" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="J4" s="41"/>
       <c r="K4" s="41" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L4" s="41"/>
       <c r="M4" s="41" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="N4" s="41" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="O4" s="41" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="P4" s="41"/>
       <c r="Q4" s="41" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="R4" s="41"/>
       <c r="S4" s="41"/>
@@ -11655,49 +11658,49 @@
     </row>
     <row r="5" ht="15.75" customHeight="1">
       <c r="A5" s="41" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C5" s="41" t="s">
         <v>71</v>
       </c>
       <c r="D5" s="41" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E5" s="43" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F5" s="42" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="G5" s="42" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H5" s="42" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I5" s="42" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="J5" s="41"/>
       <c r="K5" s="41" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L5" s="41"/>
       <c r="M5" s="41" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="N5" s="41" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="O5" s="41" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="P5" s="41"/>
       <c r="Q5" s="41" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="R5" s="41"/>
       <c r="S5" s="41"/>
@@ -11714,49 +11717,49 @@
     </row>
     <row r="6" ht="15.75" customHeight="1">
       <c r="A6" s="44" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B6" s="45" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C6" s="44" t="s">
         <v>71</v>
       </c>
       <c r="D6" s="44" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E6" s="46" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F6" s="45" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="G6" s="45" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="H6" s="45" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I6" s="42" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="J6" s="44"/>
       <c r="K6" s="44" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L6" s="44"/>
       <c r="M6" s="44" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="N6" s="44" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="O6" s="44" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="P6" s="44"/>
       <c r="Q6" s="41" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="R6" s="44"/>
       <c r="S6" s="44"/>
@@ -11773,49 +11776,49 @@
     </row>
     <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="41" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B7" s="42" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C7" s="41" t="s">
         <v>71</v>
       </c>
       <c r="D7" s="41" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E7" s="43" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F7" s="42" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="G7" s="42" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="H7" s="42" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="I7" s="42" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="J7" s="41"/>
       <c r="K7" s="41" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L7" s="41"/>
       <c r="M7" s="41" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="N7" s="41" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="O7" s="41" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="P7" s="41"/>
       <c r="Q7" s="41" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="R7" s="41"/>
       <c r="S7" s="41"/>
@@ -11832,49 +11835,49 @@
     </row>
     <row r="8" ht="15.75" customHeight="1">
       <c r="A8" s="41" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B8" s="42" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C8" s="41" t="s">
         <v>71</v>
       </c>
       <c r="D8" s="41" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E8" s="43" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F8" s="42" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="G8" s="42" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="H8" s="42" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="I8" s="42" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="J8" s="41"/>
       <c r="K8" s="41" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L8" s="41"/>
       <c r="M8" s="41" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="N8" s="41" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="O8" s="41" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="P8" s="41"/>
       <c r="Q8" s="41" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="R8" s="41"/>
       <c r="S8" s="41"/>
@@ -11891,49 +11894,49 @@
     </row>
     <row r="9" ht="15.75" customHeight="1">
       <c r="A9" s="44" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B9" s="45" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C9" s="44" t="s">
         <v>17</v>
       </c>
       <c r="D9" s="44" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E9" s="46" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F9" s="45" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="G9" s="45" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H9" s="45" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I9" s="42" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="J9" s="44"/>
       <c r="K9" s="44" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L9" s="44"/>
       <c r="M9" s="44" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="N9" s="44" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="O9" s="44" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="P9" s="44"/>
       <c r="Q9" s="41" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="R9" s="44"/>
       <c r="S9" s="44"/>
@@ -11950,47 +11953,47 @@
     </row>
     <row r="10" ht="15.75" customHeight="1">
       <c r="A10" s="47" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B10" s="47" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C10" s="48" t="s">
         <v>17</v>
       </c>
       <c r="D10" s="47" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E10" s="47" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F10" s="47" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G10" s="47" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="H10" s="49" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="I10" s="47"/>
       <c r="J10" s="47"/>
       <c r="K10" s="47" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L10" s="47"/>
       <c r="M10" s="49" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="N10" s="47" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="O10" s="49" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="P10" s="47"/>
       <c r="Q10" s="41" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="R10" s="47"/>
       <c r="S10" s="47"/>
@@ -12007,47 +12010,47 @@
     </row>
     <row r="11" ht="15.75" customHeight="1">
       <c r="A11" s="47" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B11" s="47" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C11" s="48" t="s">
         <v>71</v>
       </c>
       <c r="D11" s="47" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E11" s="47" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F11" s="47" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G11" s="47" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="H11" s="49" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="I11" s="47"/>
       <c r="J11" s="47"/>
       <c r="K11" s="47" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L11" s="47"/>
       <c r="M11" s="49" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="N11" s="47" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="O11" s="49" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="P11" s="47"/>
       <c r="Q11" s="41" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="R11" s="47"/>
       <c r="S11" s="47"/>
@@ -12064,47 +12067,47 @@
     </row>
     <row r="12" ht="15.75" customHeight="1">
       <c r="A12" s="47" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B12" s="47" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C12" s="48" t="s">
         <v>71</v>
       </c>
       <c r="D12" s="47" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E12" s="47" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F12" s="47" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G12" s="47" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="H12" s="49" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="I12" s="47"/>
       <c r="J12" s="47"/>
       <c r="K12" s="47" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L12" s="47"/>
       <c r="M12" s="49" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="N12" s="47" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="O12" s="49" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="P12" s="47"/>
       <c r="Q12" s="41" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="R12" s="47"/>
       <c r="S12" s="47"/>
@@ -12121,47 +12124,47 @@
     </row>
     <row r="13" ht="15.75" customHeight="1">
       <c r="A13" s="47" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B13" s="47" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C13" s="48" t="s">
         <v>17</v>
       </c>
       <c r="D13" s="47" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E13" s="47" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F13" s="47" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G13" s="47" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="H13" s="49" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="I13" s="47"/>
       <c r="J13" s="47"/>
       <c r="K13" s="47" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L13" s="47"/>
       <c r="M13" s="49" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="N13" s="47" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="O13" s="49" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="P13" s="47"/>
       <c r="Q13" s="41" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="R13" s="47"/>
       <c r="S13" s="47"/>
@@ -12178,47 +12181,47 @@
     </row>
     <row r="14" ht="15.75" customHeight="1">
       <c r="A14" s="47" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B14" s="47" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C14" s="48" t="s">
         <v>17</v>
       </c>
       <c r="D14" s="47" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E14" s="47" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F14" s="47" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G14" s="47" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="H14" s="49" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="I14" s="47"/>
       <c r="J14" s="47"/>
       <c r="K14" s="47" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L14" s="47"/>
       <c r="M14" s="49" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="N14" s="47" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="O14" s="49" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="P14" s="47"/>
       <c r="Q14" s="41" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="R14" s="47"/>
       <c r="S14" s="47"/>
@@ -12235,47 +12238,47 @@
     </row>
     <row r="15" ht="15.75" customHeight="1">
       <c r="A15" s="47" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B15" s="47" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C15" s="48" t="s">
         <v>17</v>
       </c>
       <c r="D15" s="47" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E15" s="47" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F15" s="47" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G15" s="47" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="H15" s="49" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="I15" s="47"/>
       <c r="J15" s="47"/>
       <c r="K15" s="47" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L15" s="47"/>
       <c r="M15" s="49" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="N15" s="47" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="O15" s="49" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="P15" s="47"/>
       <c r="Q15" s="41" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="R15" s="47"/>
       <c r="S15" s="47"/>
@@ -12292,47 +12295,47 @@
     </row>
     <row r="16" ht="15.75" customHeight="1">
       <c r="A16" s="47" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B16" s="47" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C16" s="48" t="s">
         <v>17</v>
       </c>
       <c r="D16" s="47" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E16" s="47" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F16" s="47" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G16" s="47" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="H16" s="49" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="I16" s="47"/>
       <c r="J16" s="47"/>
       <c r="K16" s="47" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L16" s="47"/>
       <c r="M16" s="49" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="N16" s="47" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="O16" s="49" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="P16" s="47"/>
       <c r="Q16" s="41" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="R16" s="47"/>
       <c r="S16" s="47"/>
@@ -12349,192 +12352,192 @@
     </row>
     <row r="17" ht="15.75" customHeight="1">
       <c r="A17" s="50" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B17" s="50" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C17" s="41" t="s">
         <v>17</v>
       </c>
       <c r="D17" s="50" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E17" s="50" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F17" s="50" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="G17" s="50" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="H17" s="51" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="J17" s="50" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="K17" s="50" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L17" s="50" t="s">
         <v>21</v>
       </c>
       <c r="M17" s="51" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="N17" s="50" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="O17" s="51" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="Q17" s="41" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="50" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B18" s="50" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C18" s="41" t="s">
         <v>17</v>
       </c>
       <c r="D18" s="50" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E18" s="50" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="F18" s="50" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="G18" s="50" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="H18" s="51" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="J18" s="50" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="K18" s="50" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L18" s="50" t="s">
         <v>21</v>
       </c>
       <c r="M18" s="51" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="N18" s="50" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="O18" s="51" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="Q18" s="41" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="19" ht="15.75" customHeight="1">
       <c r="A19" s="50" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B19" s="50" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C19" s="41" t="s">
         <v>17</v>
       </c>
       <c r="D19" s="50" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E19" s="50" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="F19" s="50" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="G19" s="50" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="H19" s="51" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="J19" s="50" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="K19" s="50" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L19" s="50" t="s">
         <v>21</v>
       </c>
       <c r="M19" s="51" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="N19" s="50" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="O19" s="51" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="Q19" s="41" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="52" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B20" s="52" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C20" s="44" t="s">
         <v>71</v>
       </c>
       <c r="D20" s="52" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E20" s="52" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="F20" s="52" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="G20" s="52" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="H20" s="52" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="I20" s="52"/>
       <c r="J20" s="52" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="K20" s="52" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L20" s="52" t="s">
         <v>21</v>
       </c>
       <c r="M20" s="53" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="N20" s="52" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="O20" s="51" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="P20" s="52"/>
       <c r="Q20" s="41" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="R20" s="52"/>
       <c r="S20" s="52"/>
@@ -12551,51 +12554,51 @@
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="54" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B21" s="54" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C21" s="41" t="s">
         <v>17</v>
       </c>
       <c r="D21" s="55" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E21" s="55" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="F21" s="54" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="G21" s="56" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="H21" s="54" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="I21" s="57" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="J21" s="58"/>
       <c r="K21" s="58" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L21" s="58"/>
       <c r="M21" s="59" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="N21" s="54" t="s">
         <v>26</v>
       </c>
       <c r="O21" s="55" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="P21" s="60" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="Q21" s="41" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="R21" s="58"/>
       <c r="S21" s="58"/>
@@ -12612,237 +12615,237 @@
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="50" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B22" s="50" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C22" s="41" t="s">
         <v>71</v>
       </c>
       <c r="D22" s="50" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E22" s="57" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="F22" s="57" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="G22" s="57" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="H22" s="61" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="I22" s="57" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="K22" s="50" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="M22" s="51" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="N22" s="50" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="O22" s="51" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="P22" s="60" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="Q22" s="41" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="50" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B23" s="50" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C23" s="41" t="s">
         <v>71</v>
       </c>
       <c r="D23" s="50" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E23" s="57" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="F23" s="62" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="G23" s="57" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="H23" s="61" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="I23" s="57" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="K23" s="50" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="M23" s="51" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="N23" s="50" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="O23" s="51" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="P23" s="60" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="Q23" s="41" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="50" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B24" s="50" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C24" s="41" t="s">
         <v>71</v>
       </c>
       <c r="D24" s="50" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E24" s="57" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="F24" s="57" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="G24" s="50" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="H24" s="61" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="I24" s="57" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="K24" s="50" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="M24" s="51" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="N24" s="50" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="O24" s="51"/>
       <c r="P24" s="60" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="Q24" s="41" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="50" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B25" s="50" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C25" s="41" t="s">
         <v>71</v>
       </c>
       <c r="D25" s="50" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E25" s="57" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="F25" s="57" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="G25" s="50" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="H25" s="41" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="I25" s="57" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="K25" s="50" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="M25" s="51" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="N25" s="50" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="O25" s="51" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="P25" s="60" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="Q25" s="41" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="52" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B26" s="52" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C26" s="44" t="s">
         <v>71</v>
       </c>
       <c r="D26" s="52" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E26" s="63" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="F26" s="63" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="G26" s="52" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="H26" s="44" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="I26" s="57" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="J26" s="52"/>
       <c r="K26" s="52" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L26" s="52"/>
       <c r="M26" s="53" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="N26" s="52" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="O26" s="53" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="P26" s="60" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="Q26" s="41" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="R26" s="52"/>
       <c r="S26" s="52"/>
@@ -12859,326 +12862,326 @@
     </row>
     <row r="27" ht="51.75" customHeight="1">
       <c r="A27" s="51" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B27" s="50" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C27" s="41" t="s">
         <v>71</v>
       </c>
       <c r="D27" s="50" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="E27" s="50" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="F27" s="50" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="G27" s="50" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="H27" s="51" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="K27" s="50" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="M27" s="51" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="N27" s="50" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="O27" s="51" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="Q27" s="41" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="28" ht="66.75" customHeight="1">
       <c r="A28" s="50" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B28" s="50" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C28" s="41" t="s">
         <v>71</v>
       </c>
       <c r="D28" s="50" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="E28" s="50" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="F28" s="50" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="G28" s="50" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="H28" s="51" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="K28" s="50" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="M28" s="51" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="N28" s="50" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="O28" s="51" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="Q28" s="41" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="29" ht="46.5" customHeight="1">
       <c r="A29" s="50" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B29" s="50" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C29" s="41" t="s">
         <v>17</v>
       </c>
       <c r="D29" s="50" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="E29" s="50" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="F29" s="50" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="G29" s="50" t="s">
         <v>21</v>
       </c>
       <c r="H29" s="51" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="K29" s="50" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="M29" s="51" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="N29" s="50" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="O29" s="51" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="Q29" s="41" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="50" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B30" s="50" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C30" s="41" t="s">
         <v>17</v>
       </c>
       <c r="D30" s="50" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="E30" s="50" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="F30" s="50" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="G30" s="50" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="H30" s="61" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="K30" s="50" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="M30" s="51" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="O30" s="51" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="Q30" s="41" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="50" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B31" s="50" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C31" s="41" t="s">
         <v>17</v>
       </c>
       <c r="D31" s="50" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="E31" s="50" t="s">
         <v>21</v>
       </c>
       <c r="F31" s="50" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="G31" s="50" t="s">
         <v>21</v>
       </c>
       <c r="H31" s="61" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="K31" s="50" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="M31" s="51" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="O31" s="51" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="Q31" s="41" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="50" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B32" s="50" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="C32" s="41" t="s">
         <v>17</v>
       </c>
       <c r="D32" s="50" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E32" s="50" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="F32" s="50" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="G32" s="50" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="H32" s="61" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="I32" s="64" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="J32" s="50" t="s">
         <v>21</v>
       </c>
       <c r="K32" s="50" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="M32" s="51" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="O32" s="51" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="Q32" s="41" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="33" ht="55.5" customHeight="1">
       <c r="A33" s="50" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="B33" s="50" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C33" s="41" t="s">
         <v>17</v>
       </c>
       <c r="D33" s="50" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="E33" s="50" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="F33" s="50" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="G33" s="65" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="H33" s="61" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="J33" s="50" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="K33" s="50" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="M33" s="51" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="N33" s="50" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="O33" s="51" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="Q33" s="41" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="34" ht="63.75" customHeight="1">
       <c r="A34" s="66" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B34" s="50" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="C34" s="41" t="s">
         <v>71</v>
       </c>
       <c r="D34" s="50" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E34" s="66" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="F34" s="66" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="G34" s="66" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="H34" s="67" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="I34" s="66"/>
       <c r="J34" s="66" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="K34" s="50" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L34" s="66"/>
       <c r="M34" s="68" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="N34" s="66" t="s">
         <v>26</v>
@@ -13188,7 +13191,7 @@
       </c>
       <c r="P34" s="66"/>
       <c r="Q34" s="41" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="R34" s="66"/>
       <c r="S34" s="66"/>
@@ -13205,39 +13208,39 @@
     </row>
     <row r="35" ht="67.5" customHeight="1">
       <c r="A35" s="66" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="B35" s="50" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="C35" s="41" t="s">
         <v>71</v>
       </c>
       <c r="D35" s="50" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E35" s="66" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="F35" s="66" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="G35" s="66" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="H35" s="67" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="I35" s="66"/>
       <c r="J35" s="66" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="K35" s="50" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L35" s="66"/>
       <c r="M35" s="68" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="N35" s="66" t="s">
         <v>26</v>
@@ -13247,7 +13250,7 @@
       </c>
       <c r="P35" s="66"/>
       <c r="Q35" s="41" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="R35" s="66"/>
       <c r="S35" s="66"/>
@@ -13264,37 +13267,37 @@
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="50" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B36" s="50" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="C36" s="41" t="s">
         <v>17</v>
       </c>
       <c r="D36" s="50" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E36" s="69" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="F36" s="50" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="G36" s="50" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="H36" s="51" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="J36" s="50" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="K36" s="50" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="M36" s="70" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="N36" s="50" t="s">
         <v>26</v>
@@ -13303,54 +13306,54 @@
         <v>27</v>
       </c>
       <c r="Q36" s="41" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="66" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B37" s="66" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="C37" s="41" t="s">
         <v>17</v>
       </c>
       <c r="D37" s="66" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E37" s="64" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="F37" s="66" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="G37" s="66" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="H37" s="71" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="I37" s="66"/>
       <c r="J37" s="66" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="K37" s="50" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L37" s="66"/>
       <c r="M37" s="68" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="N37" s="66" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="O37" s="67" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="P37" s="66"/>
       <c r="Q37" s="41" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="R37" s="66"/>
       <c r="S37" s="66"/>
@@ -13367,49 +13370,49 @@
     </row>
     <row r="38" ht="15.75" customHeight="1">
       <c r="A38" s="66" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B38" s="66" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="C38" s="41" t="s">
         <v>71</v>
       </c>
       <c r="D38" s="66" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E38" s="64" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="F38" s="66" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="G38" s="66" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="H38" s="71" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="I38" s="66"/>
       <c r="J38" s="66" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="K38" s="66" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L38" s="66"/>
       <c r="M38" s="68" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="N38" s="66" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="O38" s="67" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="P38" s="66"/>
       <c r="Q38" s="41" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="R38" s="66"/>
       <c r="S38" s="66"/>

</xml_diff>